<commit_message>
Completed the __init__ tests and ran all four of them
</commit_message>
<xml_diff>
--- a/tests/A02_pixell_test_plan_chequing_account.xlsx
+++ b/tests/A02_pixell_test_plan_chequing_account.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lauri\Desktop\Intermediate Software Development0315\2. Assignments\assignments\assignment_02\instructions\given_files\assignment_2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ab840a8a6702860f/Documentos/RRC_Term2/intermediate_software_development/project/isd_project/tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2873F10E-F8B1-4F89-8CDF-A98B96DD770E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="62" documentId="13_ncr:1_{2873F10E-F8B1-4F89-8CDF-A98B96DD770E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6EEEF2F2-53F4-4A32-B107-55F31C6B21DA}"/>
   <bookViews>
-    <workbookView xWindow="2640" yWindow="3555" windowWidth="25185" windowHeight="11415" xr2:uid="{8D9DD509-55B1-455D-8036-16809AD15960}"/>
+    <workbookView xWindow="-17400" yWindow="0" windowWidth="17505" windowHeight="15585" xr2:uid="{8D9DD509-55B1-455D-8036-16809AD15960}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -183,7 +183,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="33">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -249,6 +249,59 @@
   </si>
   <si>
     <t>Attributes are set to input values (ensure to test for superclass and subclass attributes)</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>Amanda Dadalt Makino</t>
+  </si>
+  <si>
+    <t>Attributes set</t>
+  </si>
+  <si>
+    <t>overdraft_limit = -100</t>
+  </si>
+  <si>
+    <t>ChequingAccount(1234, 4567, 10000, (2024,11,14), 200.0, 10.0)</t>
+  </si>
+  <si>
+    <t>account_number = 1234
+client_number = 4567
+balance = 10000
+date_created = (2024, 11, 14)
+overdraft_limit = 200.0
+overdraft_rate = 10.0</t>
+  </si>
+  <si>
+    <t>account_number = 1234
+client_number = 4567
+balance = 10000
+date_created = 
+overdraft_limit = 200.0
+overdraft_rate = 10.0</t>
+  </si>
+  <si>
+    <t>overdraft_rate = 0.05</t>
+  </si>
+  <si>
+    <t>account_number = 1234
+client_number = 4567
+balance = 10000
+date_created = (2024, 11, 14)
+overdraft_limit = "hundred"
+overdraft_rate = 10.0</t>
+  </si>
+  <si>
+    <t>account_number = 1234
+client_number = 4567
+balance = 10000
+date_created = (2024, 11, 14)
+overdraft_limit = 200.0
+overdraft_rate = "ten"</t>
+  </si>
+  <si>
+    <t>Account Number: 1234 Balance: $10.000 Overdraft Limit: $100.00 Overdraft Rate: 10% Account Type: Chequing</t>
   </si>
 </sst>
 </file>
@@ -755,6 +808,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1153,18 +1210,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DADEBCC4-BB44-48CD-B9AB-1E2FD3EE0EEB}">
   <dimension ref="B1:G32"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="12.7109375" customWidth="1"/>
-    <col min="3" max="3" width="22.28515625" customWidth="1"/>
-    <col min="4" max="4" width="32.7109375" customWidth="1"/>
-    <col min="5" max="5" width="31.5703125" customWidth="1"/>
-    <col min="6" max="6" width="28.28515625" customWidth="1"/>
-    <col min="7" max="7" width="48.42578125" customWidth="1"/>
+    <col min="2" max="2" width="12.6640625" customWidth="1"/>
+    <col min="3" max="3" width="22.33203125" customWidth="1"/>
+    <col min="4" max="4" width="32.6640625" customWidth="1"/>
+    <col min="5" max="5" width="31.5546875" customWidth="1"/>
+    <col min="6" max="6" width="29.44140625" customWidth="1"/>
+    <col min="7" max="7" width="43.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="2:7" ht="73.150000000000006" customHeight="1" thickBot="1" x14ac:dyDescent="1.45">
+    <row r="1" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="2:7" ht="73.2" customHeight="1" thickBot="1" x14ac:dyDescent="1.8">
       <c r="B2" s="2" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
@@ -1176,14 +1233,16 @@
       <c r="F2" s="15"/>
       <c r="G2" s="15"/>
     </row>
-    <row r="3" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="16"/>
+      <c r="C3" s="16" t="s">
+        <v>23</v>
+      </c>
       <c r="D3" s="17"/>
     </row>
-    <row r="4" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B4" s="7" t="s">
         <v>3</v>
       </c>
@@ -1192,10 +1251,10 @@
       </c>
       <c r="D4" s="19"/>
     </row>
-    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B5" s="1"/>
     </row>
-    <row r="6" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B6" s="8" t="s">
         <v>0</v>
       </c>
@@ -1215,7 +1274,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:7" ht="94.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B7" s="11">
         <v>1</v>
       </c>
@@ -1225,11 +1284,17 @@
       <c r="D7" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="E7" s="12"/>
-      <c r="F7" s="12"/>
-      <c r="G7" s="12"/>
-    </row>
-    <row r="8" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E7" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="F7" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="G7" s="12" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="2:7" ht="93" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B8" s="3">
         <v>2</v>
       </c>
@@ -1239,11 +1304,17 @@
       <c r="D8" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="12"/>
-      <c r="F8" s="12"/>
-      <c r="G8" s="12"/>
-    </row>
-    <row r="9" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E8" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="F8" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="G8" s="12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="2:7" ht="93" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B9" s="11">
         <v>3</v>
       </c>
@@ -1253,11 +1324,17 @@
       <c r="D9" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="E9" s="12"/>
-      <c r="F9" s="13"/>
-      <c r="G9" s="12"/>
-    </row>
-    <row r="10" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E9" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="F9" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="G9" s="12" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="10" spans="2:7" ht="94.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="11">
         <v>4</v>
       </c>
@@ -1267,11 +1344,15 @@
       <c r="D10" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="E10" s="13"/>
-      <c r="F10" s="13"/>
+      <c r="E10" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="F10" s="13" t="s">
+        <v>28</v>
+      </c>
       <c r="G10" s="13"/>
     </row>
-    <row r="11" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:7" ht="37.799999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B11" s="3">
         <v>5</v>
       </c>
@@ -1281,11 +1362,15 @@
       <c r="D11" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E11" s="12"/>
-      <c r="F11" s="13"/>
+      <c r="E11" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="F11" s="13" t="s">
+        <v>22</v>
+      </c>
       <c r="G11" s="13"/>
     </row>
-    <row r="12" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:7" ht="39.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B12" s="11">
         <v>6</v>
       </c>
@@ -1295,11 +1380,15 @@
       <c r="D12" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="E12" s="13"/>
-      <c r="F12" s="13"/>
+      <c r="E12" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="F12" s="13" t="s">
+        <v>22</v>
+      </c>
       <c r="G12" s="13"/>
     </row>
-    <row r="13" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:7" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="11">
         <v>7</v>
       </c>
@@ -1309,11 +1398,15 @@
       <c r="D13" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E13" s="12"/>
-      <c r="F13" s="13"/>
+      <c r="E13" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="F13" s="13" t="s">
+        <v>22</v>
+      </c>
       <c r="G13" s="13"/>
     </row>
-    <row r="14" spans="2:7" ht="58.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:7" ht="49.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B14" s="3">
         <v>8</v>
       </c>
@@ -1323,11 +1416,17 @@
       <c r="D14" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E14" s="12"/>
-      <c r="F14" s="13"/>
-      <c r="G14" s="13"/>
-    </row>
-    <row r="15" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E14" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="F14" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="G14" s="13" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="15" spans="2:7" ht="31.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B15" s="11">
         <v>9</v>
       </c>
@@ -1337,7 +1436,7 @@
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
     </row>
-    <row r="16" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:7" ht="31.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="11">
         <v>10</v>
       </c>
@@ -1347,7 +1446,7 @@
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
     </row>
-    <row r="17" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:7" ht="31.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B17" s="3">
         <v>11</v>
       </c>
@@ -1357,7 +1456,7 @@
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
     </row>
-    <row r="18" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:7" ht="31.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B18" s="11">
         <v>12</v>
       </c>
@@ -1367,7 +1466,7 @@
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
     </row>
-    <row r="19" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:7" ht="31.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="11">
         <v>13</v>
       </c>
@@ -1377,7 +1476,7 @@
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
     </row>
-    <row r="20" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:7" ht="31.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B20" s="3">
         <v>14</v>
       </c>
@@ -1387,7 +1486,7 @@
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
     </row>
-    <row r="21" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:7" ht="31.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B21" s="11">
         <v>15</v>
       </c>
@@ -1397,7 +1496,7 @@
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
     </row>
-    <row r="22" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:7" ht="31.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B22" s="11">
         <v>16</v>
       </c>
@@ -1407,7 +1506,7 @@
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
     </row>
-    <row r="23" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:7" ht="31.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B23" s="3">
         <v>17</v>
       </c>
@@ -1417,7 +1516,7 @@
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
     </row>
-    <row r="24" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:7" ht="31.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B24" s="11">
         <v>18</v>
       </c>
@@ -1427,7 +1526,7 @@
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
     </row>
-    <row r="25" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:7" ht="31.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B25" s="11">
         <v>19</v>
       </c>
@@ -1437,7 +1536,7 @@
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
     </row>
-    <row r="26" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:7" ht="31.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B26" s="3">
         <v>20</v>
       </c>
@@ -1447,7 +1546,7 @@
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
     </row>
-    <row r="27" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:7" ht="31.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B27" s="11">
         <v>21</v>
       </c>
@@ -1457,7 +1556,7 @@
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
     </row>
-    <row r="28" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:7" ht="31.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B28" s="11">
         <v>22</v>
       </c>
@@ -1467,7 +1566,7 @@
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
     </row>
-    <row r="29" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:7" ht="31.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B29" s="3">
         <v>23</v>
       </c>
@@ -1477,7 +1576,7 @@
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
     </row>
-    <row r="30" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:7" ht="31.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B30" s="11">
         <v>24</v>
       </c>
@@ -1487,7 +1586,7 @@
       <c r="F30" s="5"/>
       <c r="G30" s="5"/>
     </row>
-    <row r="32" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B32" s="20" t="s">
         <v>6</v>
       </c>

</xml_diff>

<commit_message>
Ran all three tests for the get_services_charge method
</commit_message>
<xml_diff>
--- a/tests/A02_pixell_test_plan_chequing_account.xlsx
+++ b/tests/A02_pixell_test_plan_chequing_account.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ab840a8a6702860f/Documentos/RRC_Term2/intermediate_software_development/project/isd_project/tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="62" documentId="13_ncr:1_{2873F10E-F8B1-4F89-8CDF-A98B96DD770E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6EEEF2F2-53F4-4A32-B107-55F31C6B21DA}"/>
+  <xr:revisionPtr revIDLastSave="75" documentId="13_ncr:1_{2873F10E-F8B1-4F89-8CDF-A98B96DD770E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4B604E1C-667D-4E70-AA58-E737FC4CCB4F}"/>
   <bookViews>
     <workbookView xWindow="-17400" yWindow="0" windowWidth="17505" windowHeight="15585" xr2:uid="{8D9DD509-55B1-455D-8036-16809AD15960}"/>
   </bookViews>
@@ -183,7 +183,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="36">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -274,14 +274,6 @@
 overdraft_rate = 10.0</t>
   </si>
   <si>
-    <t>account_number = 1234
-client_number = 4567
-balance = 10000
-date_created = 
-overdraft_limit = 200.0
-overdraft_rate = 10.0</t>
-  </si>
-  <si>
     <t>overdraft_rate = 0.05</t>
   </si>
   <si>
@@ -303,11 +295,31 @@
   <si>
     <t>Account Number: 1234 Balance: $10.000 Overdraft Limit: $100.00 Overdraft Rate: 10% Account Type: Chequing</t>
   </si>
+  <si>
+    <t>account_number = 1234
+client_number = 4567
+balance = 10000
+date_created = "November 14"
+overdraft_limit = 200.0
+overdraft_rate = 10.0</t>
+  </si>
+  <si>
+    <t>current date</t>
+  </si>
+  <si>
+    <t>ChequingAccount(1234, 4567, 100, (2024,11,14), 200.0, 10.0)</t>
+  </si>
+  <si>
+    <t>ChequingAccount(1234, 4567, 200, (2024,11,14), 200.0, 10.0)</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00;[Red]\-&quot;$&quot;#,##0.00"/>
+  </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -608,7 +620,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
@@ -662,6 +674,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="8" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1308,7 +1323,7 @@
         <v>22</v>
       </c>
       <c r="F8" s="12" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G8" s="12" t="s">
         <v>25</v>
@@ -1328,10 +1343,10 @@
         <v>22</v>
       </c>
       <c r="F9" s="13" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G9" s="12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10" spans="2:7" ht="94.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1348,9 +1363,11 @@
         <v>22</v>
       </c>
       <c r="F10" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="G10" s="13"/>
+        <v>32</v>
+      </c>
+      <c r="G10" s="13" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="11" spans="2:7" ht="37.799999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B11" s="3">
@@ -1368,7 +1385,9 @@
       <c r="F11" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="G11" s="13"/>
+      <c r="G11" s="22">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="12" spans="2:7" ht="39.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B12" s="11">
@@ -1381,12 +1400,14 @@
         <v>18</v>
       </c>
       <c r="E12" s="13" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="F12" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="G12" s="13"/>
+      <c r="G12" s="13">
+        <v>1000.5</v>
+      </c>
     </row>
     <row r="13" spans="2:7" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="11">
@@ -1399,12 +1420,14 @@
         <v>19</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="F13" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="G13" s="13"/>
+      <c r="G13" s="22">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="14" spans="2:7" ht="49.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B14" s="3">
@@ -1423,7 +1446,7 @@
         <v>22</v>
       </c>
       <c r="G14" s="13" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="15" spans="2:7" ht="31.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Completed both tests for the str methods and ran successfully
</commit_message>
<xml_diff>
--- a/tests/A02_pixell_test_plan_chequing_account.xlsx
+++ b/tests/A02_pixell_test_plan_chequing_account.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ab840a8a6702860f/Documentos/RRC_Term2/intermediate_software_development/project/isd_project/tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="75" documentId="13_ncr:1_{2873F10E-F8B1-4F89-8CDF-A98B96DD770E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4B604E1C-667D-4E70-AA58-E737FC4CCB4F}"/>
+  <xr:revisionPtr revIDLastSave="77" documentId="13_ncr:1_{2873F10E-F8B1-4F89-8CDF-A98B96DD770E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D9162FB1-D255-48A8-9247-F4EDCCF08CA5}"/>
   <bookViews>
-    <workbookView xWindow="-17400" yWindow="0" windowWidth="17505" windowHeight="15585" xr2:uid="{8D9DD509-55B1-455D-8036-16809AD15960}"/>
+    <workbookView xWindow="-14505" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{8D9DD509-55B1-455D-8036-16809AD15960}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -293,9 +293,6 @@
 overdraft_rate = "ten"</t>
   </si>
   <si>
-    <t>Account Number: 1234 Balance: $10.000 Overdraft Limit: $100.00 Overdraft Rate: 10% Account Type: Chequing</t>
-  </si>
-  <si>
     <t>account_number = 1234
 client_number = 4567
 balance = 10000
@@ -311,6 +308,9 @@
   </si>
   <si>
     <t>ChequingAccount(1234, 4567, 200, (2024,11,14), 200.0, 10.0)</t>
+  </si>
+  <si>
+    <t>Account Number: 1234 Balance: $10.000.00 Overdraft Limit: $200.00 Overdraft Rate: 10% Account Type: Chequing</t>
   </si>
 </sst>
 </file>
@@ -651,6 +651,9 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="8" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -674,9 +677,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="8" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1232,7 +1232,7 @@
     <col min="4" max="4" width="32.6640625" customWidth="1"/>
     <col min="5" max="5" width="31.5546875" customWidth="1"/>
     <col min="6" max="6" width="29.44140625" customWidth="1"/>
-    <col min="7" max="7" width="43.5546875" customWidth="1"/>
+    <col min="7" max="7" width="40.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
@@ -1240,31 +1240,31 @@
       <c r="B2" s="2" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="C2" s="14" t="s">
+      <c r="C2" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
     </row>
     <row r="3" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="16" t="s">
+      <c r="C3" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="D3" s="17"/>
+      <c r="D3" s="18"/>
     </row>
     <row r="4" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B4" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="19"/>
+      <c r="D4" s="20"/>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B5" s="1"/>
@@ -1363,10 +1363,10 @@
         <v>22</v>
       </c>
       <c r="F10" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="G10" s="13" t="s">
         <v>32</v>
-      </c>
-      <c r="G10" s="13" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="11" spans="2:7" ht="37.799999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -1385,7 +1385,7 @@
       <c r="F11" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="G11" s="22">
+      <c r="G11" s="14">
         <v>0.5</v>
       </c>
     </row>
@@ -1400,7 +1400,7 @@
         <v>18</v>
       </c>
       <c r="E12" s="13" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F12" s="13" t="s">
         <v>22</v>
@@ -1420,12 +1420,12 @@
         <v>19</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F13" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="G13" s="22">
+      <c r="G13" s="14">
         <v>0.5</v>
       </c>
     </row>
@@ -1446,7 +1446,7 @@
         <v>22</v>
       </c>
       <c r="G14" s="13" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="15" spans="2:7" ht="31.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -1610,14 +1610,14 @@
       <c r="G30" s="5"/>
     </row>
     <row r="32" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B32" s="20" t="s">
+      <c r="B32" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="C32" s="21"/>
-      <c r="D32" s="21"/>
-      <c r="E32" s="21"/>
-      <c r="F32" s="21"/>
-      <c r="G32" s="21"/>
+      <c r="C32" s="22"/>
+      <c r="D32" s="22"/>
+      <c r="E32" s="22"/>
+      <c r="F32" s="22"/>
+      <c r="G32" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>